<commit_message>
Atualiza produtos pelo painel
</commit_message>
<xml_diff>
--- a/produtos.xlsx
+++ b/produtos.xlsx
@@ -33,9 +33,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="&quot;R$&quot; #,##0.00"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -66,9 +65,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -400,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="32.83203125" customWidth="1"/>
@@ -438,35 +436,9 @@
         <v>Foto</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Sim</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Inseticida Poderoso</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v>500</v>
-      </c>
-      <c r="E2" s="1">
-        <v>16.49</v>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v>inseticida-poderoso-mv5g0p56.jpg</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -496,7 +468,7 @@
         <v>WhatsApp</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>5581999180003</v>
       </c>
       <c r="C2" t="str">
         <v>Só números, com 55 + DDD</v>
@@ -529,7 +501,7 @@
         <v>Endereço</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>Avenida B nº 5 Loja C, Maranguape II, Paulista-PE, CEP,:53.421-036</v>
       </c>
       <c r="C5" t="str">
         <v>Aparece na seção Contato do site</v>

</xml_diff>